<commit_message>
Update dividend calendar 2026-09-14
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 09/07/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 09/14/2026</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-224</v>
+        <v>-231</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06045694038225009</v>
+        <v>0.0618816332174422</v>
       </c>
     </row>
     <row r="7">
@@ -726,7 +726,7 @@
         <v>46263</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>-9</v>
+        <v>-16</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46662</v>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.03239186184874104</v>
+        <v>0.03249306950164277</v>
       </c>
     </row>
     <row r="8">
@@ -771,11 +771,11 @@
       <c r="H8" s="10" t="n">
         <v>46278</v>
       </c>
-      <c r="I8" s="13" t="n">
-        <v>6</v>
+      <c r="I8" s="11" t="n">
+        <v>-1</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>46344</v>
+        <v>46709</v>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.007284370444425581</v>
+        <v>0.007252874320868801</v>
       </c>
     </row>
     <row r="9">
@@ -818,7 +818,7 @@
         <v>46280</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46668</v>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.05648185150526099</v>
+        <v>0.05532352119915055</v>
       </c>
     </row>
     <row r="10">
@@ -864,7 +864,7 @@
         <v>46285</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46325</v>
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.0219780217704021</v>
+        <v>0.02153962736846832</v>
       </c>
     </row>
     <row r="11">
@@ -910,7 +910,7 @@
         <v>46305</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46339</v>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.02866320644948689</v>
+        <v>0.028948135474036</v>
       </c>
     </row>
     <row r="12">
@@ -956,7 +956,7 @@
         <v>46311</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46386</v>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.01143105184521834</v>
+        <v>0.0127142515706196</v>
       </c>
     </row>
     <row r="13">
@@ -1002,7 +1002,7 @@
         <v>46318</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46352</v>
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.01930542489909123</v>
+        <v>0.01974143087025879</v>
       </c>
     </row>
     <row r="14">
@@ -1048,7 +1048,7 @@
         <v>46322</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46338</v>
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.0238650142641304</v>
+        <v>0.02491484184914842</v>
       </c>
     </row>
     <row r="15">
@@ -1094,7 +1094,7 @@
         <v>46329</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46338</v>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.007251850465255884</v>
+        <v>0.007397361552028218</v>
       </c>
     </row>
     <row r="16">
@@ -1140,7 +1140,7 @@
         <v>46332</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46346</v>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.02548302872062663</v>
+        <v>0.02583787857341831</v>
       </c>
     </row>
     <row r="17">
@@ -1186,7 +1186,7 @@
         <v>46341</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46340</v>
@@ -1197,7 +1197,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.02583558016217738</v>
+        <v>0.02451651249736115</v>
       </c>
     </row>
     <row r="18">
@@ -1232,7 +1232,7 @@
         <v>46344</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46385</v>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.03686635815083875</v>
+        <v>0.03748535638894003</v>
       </c>
     </row>
     <row r="19">
@@ -1278,7 +1278,7 @@
         <v>46347</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46358</v>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.04270833163625671</v>
+        <v>0.04430037762617224</v>
       </c>
     </row>
     <row r="20">
@@ -1324,7 +1324,7 @@
         <v>46352</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J20" s="10" t="n">
         <v>46400</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0.05441039694455867</v>
+        <v>0.05595607625096392</v>
       </c>
     </row>
     <row r="21">
@@ -1370,7 +1370,7 @@
         <v>46360</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46371</v>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.04719763849938742</v>
+        <v>0.04971885038416789</v>
       </c>
     </row>
     <row r="22">
@@ -1416,7 +1416,7 @@
         <v>46366</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46432</v>
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.02305422717269788</v>
+        <v>0.02668498548328576</v>
       </c>
     </row>
     <row r="23">
@@ -1462,7 +1462,7 @@
         <v>46380</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46436</v>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.02419964820546709</v>
+        <v>0.02463433333150609</v>
       </c>
     </row>
     <row r="24">
@@ -1508,7 +1508,7 @@
         <v>46383</v>
       </c>
       <c r="I24" s="21" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="J24" s="20" t="n">
         <v>46404</v>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="L24" s="19" t="n">
-        <v>0.01515151568586133</v>
+        <v>0.01539665983034154</v>
       </c>
     </row>
     <row r="25">
@@ -1554,7 +1554,7 @@
         <v>46402</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46483</v>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.014506198907202</v>
+        <v>0.01446715458684541</v>
       </c>
     </row>
     <row r="26">
@@ -1600,7 +1600,7 @@
         <v>46411</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46435</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.03841005375174777</v>
+        <v>0.03957219387294963</v>
       </c>
     </row>
     <row r="27">
@@ -1646,7 +1646,7 @@
         <v>46417</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="J27" s="10" t="n">
         <v>46433</v>
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="L27" s="9" t="n">
-        <v>0.03413230964368608</v>
+        <v>0.03291115891894363</v>
       </c>
     </row>
     <row r="28">
@@ -1692,7 +1692,7 @@
         <v>46423</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46473</v>
@@ -1703,7 +1703,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.02484978622141126</v>
+        <v>0.02673438847314084</v>
       </c>
     </row>
     <row r="29">
@@ -1738,7 +1738,7 @@
         <v>46428</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46452</v>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.01473074142109956</v>
+        <v>0.01462479053918474</v>
       </c>
     </row>
     <row r="30">
@@ -1784,7 +1784,7 @@
         <v>46428</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46460</v>
@@ -1795,7 +1795,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.04736746272382592</v>
+        <v>0.04881483149978388</v>
       </c>
     </row>
     <row r="31">
@@ -1830,7 +1830,7 @@
         <v>46429</v>
       </c>
       <c r="I31" s="21" t="n">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J31" s="20" t="n">
         <v>46450</v>
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="L31" s="19" t="n">
-        <v>0.02637130929027715</v>
+        <v>0.02641310047223251</v>
       </c>
     </row>
     <row r="32">
@@ -1876,7 +1876,7 @@
         <v>46431</v>
       </c>
       <c r="I32" s="14" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46480</v>
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.01538461581456155</v>
+        <v>0.01520224384693243</v>
       </c>
     </row>
     <row r="33">
@@ -1922,7 +1922,7 @@
         <v>46432</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46455</v>
@@ -1933,7 +1933,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.03636363786937607</v>
+        <v>0.03727399086403899</v>
       </c>
     </row>
     <row r="34">
@@ -1968,7 +1968,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46425</v>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.004986937847341924</v>
+        <v>0.005338793701200471</v>
       </c>
     </row>
     <row r="35">
@@ -2014,7 +2014,7 @@
         <v>46433</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46383</v>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.0184862591703806</v>
+        <v>0.0186580544393274</v>
       </c>
     </row>
     <row r="36">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D36" s="7" t="n">
@@ -2060,10 +2060,10 @@
         <v>46433</v>
       </c>
       <c r="I36" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J36" s="10" t="n">
-        <v>46368</v>
+        <v>46458</v>
       </c>
       <c r="K36" s="12" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.02663337418694604</v>
+        <v>0.02508574153301707</v>
       </c>
     </row>
     <row r="37">
@@ -2106,7 +2106,7 @@
         <v>46433</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46634</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.02879670887223125</v>
+        <v>0.02863412689310154</v>
       </c>
     </row>
     <row r="38">
@@ -2152,7 +2152,7 @@
         <v>46433</v>
       </c>
       <c r="I38" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46608</v>
@@ -2163,7 +2163,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.03308411372219163</v>
+        <v>0.03364219619018467</v>
       </c>
     </row>
     <row r="39">
@@ -2198,7 +2198,7 @@
         <v>46440</v>
       </c>
       <c r="I39" s="14" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46450</v>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.00883876829813468</v>
+        <v>0.00946320755973527</v>
       </c>
     </row>
     <row r="40">
@@ -2244,7 +2244,7 @@
         <v>46441</v>
       </c>
       <c r="I40" s="14" t="n">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46456</v>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.02902974724923542</v>
+        <v>0.03000740561476674</v>
       </c>
     </row>
     <row r="41">
@@ -2290,7 +2290,7 @@
         <v>46452</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46487</v>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.01769665194015332</v>
+        <v>0.01779070791836802</v>
       </c>
     </row>
     <row r="42">
@@ -2336,7 +2336,7 @@
         <v>46461</v>
       </c>
       <c r="I42" s="14" t="n">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46300</v>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.01672986770838049</v>
+        <v>0.01699235314722998</v>
       </c>
     </row>
     <row r="43">
@@ -2382,7 +2382,7 @@
         <v>46461</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46386</v>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.05309387755102041</v>
+        <v>0.05447236111291268</v>
       </c>
     </row>
     <row r="44">
@@ -2428,7 +2428,7 @@
         <v>46488</v>
       </c>
       <c r="I44" s="14" t="n">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46498</v>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.02974597055024585</v>
+        <v>0.02964170822323141</v>
       </c>
     </row>
     <row r="45">
@@ -2474,7 +2474,7 @@
         <v>46492</v>
       </c>
       <c r="I45" s="14" t="n">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="J45" s="10" t="n">
         <v>46501</v>
@@ -2485,7 +2485,7 @@
         </is>
       </c>
       <c r="L45" s="9" t="n">
-        <v>0.02008928571428572</v>
+        <v>0.0204202028393521</v>
       </c>
     </row>
     <row r="46">
@@ -2520,7 +2520,7 @@
         <v>46492</v>
       </c>
       <c r="I46" s="14" t="n">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46376</v>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.04397787742467318</v>
+        <v>0.04231333292565891</v>
       </c>
     </row>
     <row r="47">
@@ -2566,7 +2566,7 @@
         <v>46493</v>
       </c>
       <c r="I47" s="14" t="n">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46531</v>
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.01947462044851735</v>
+        <v>0.01990567170011602</v>
       </c>
     </row>
     <row r="48">
@@ -2612,7 +2612,7 @@
         <v>46499</v>
       </c>
       <c r="I48" s="14" t="n">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46526</v>
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.01991454025218246</v>
+        <v>0.01924971624665003</v>
       </c>
     </row>
     <row r="49">
@@ -2658,7 +2658,7 @@
         <v>46504</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46562</v>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.04520098596940841</v>
+        <v>0.04570717428878286</v>
       </c>
     </row>
     <row r="50">
@@ -2704,7 +2704,7 @@
         <v>46508</v>
       </c>
       <c r="I50" s="14" t="n">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46518</v>
@@ -2715,7 +2715,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.03910935860492718</v>
+        <v>0.04061086969695727</v>
       </c>
     </row>
     <row r="51">
@@ -2750,7 +2750,7 @@
         <v>46515</v>
       </c>
       <c r="I51" s="14" t="n">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46542</v>
@@ -2761,7 +2761,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.0430138762622343</v>
+        <v>0.04294834704934376</v>
       </c>
     </row>
     <row r="52">
@@ -2796,7 +2796,7 @@
         <v>46532</v>
       </c>
       <c r="I52" s="14" t="n">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46563</v>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.03058298880746655</v>
+        <v>0.03080872803355954</v>
       </c>
     </row>
     <row r="53">
@@ -2842,7 +2842,7 @@
         <v>46589</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46629</v>
@@ -2853,7 +2853,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.01961190558580643</v>
+        <v>0.0199424192610679</v>
       </c>
     </row>
     <row r="54">
@@ -2873,25 +2873,25 @@
         </is>
       </c>
       <c r="D54" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E54" s="7" t="n">
         <v>0.83</v>
       </c>
-      <c r="E54" s="7" t="n">
-        <v>0.82</v>
-      </c>
       <c r="F54" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.01204819277108435</v>
       </c>
       <c r="G54" s="9" t="n">
         <v>0.04</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>46592</v>
+        <v>46591</v>
       </c>
       <c r="I54" s="14" t="n">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="J54" s="10" t="n">
-        <v>46632</v>
+        <v>46633</v>
       </c>
       <c r="K54" s="12" t="inlineStr">
         <is>
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.03410024629403103</v>
+        <v>0.03791041525582833</v>
       </c>
     </row>
     <row r="55">
@@ -2934,7 +2934,7 @@
         <v>46594</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46613</v>
@@ -2945,7 +2945,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.01547755333783219</v>
+        <v>0.01568376395018629</v>
       </c>
     </row>
     <row r="56">
@@ -2980,7 +2980,7 @@
         <v>46595</v>
       </c>
       <c r="I56" s="14" t="n">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46614</v>
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.02466960386438792</v>
+        <v>0.0250789461211513</v>
       </c>
     </row>
     <row r="57">
@@ -3026,7 +3026,7 @@
         <v>46597</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46611</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.05372877854259377</v>
+        <v>0.05629362775477879</v>
       </c>
     </row>
     <row r="58">
@@ -3072,7 +3072,7 @@
         <v>46598</v>
       </c>
       <c r="I58" s="14" t="n">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="J58" s="10" t="n">
         <v>46629</v>
@@ -3083,7 +3083,7 @@
         </is>
       </c>
       <c r="L58" s="9" t="n">
-        <v>0.02533513789021478</v>
+        <v>0.02503037574256811</v>
       </c>
     </row>
   </sheetData>
@@ -3118,7 +3118,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 09/07/2026</t>
+          <t>Expected Increase Announcements by Month - 09/14/2026</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
         <v>46278</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>46344</v>
+        <v>46709</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>0.91</v>
@@ -4164,7 +4164,7 @@
         <v>46433</v>
       </c>
       <c r="C57" s="10" t="n">
-        <v>46368</v>
+        <v>46458</v>
       </c>
       <c r="D57" s="7" t="n">
         <v>0.32</v>
@@ -4749,16 +4749,16 @@
         </is>
       </c>
       <c r="B87" s="10" t="n">
-        <v>46592</v>
+        <v>46591</v>
       </c>
       <c r="C87" s="10" t="n">
-        <v>46632</v>
+        <v>46633</v>
       </c>
       <c r="D87" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.01204819277108435</v>
       </c>
       <c r="F87" s="12" t="inlineStr">
         <is>
@@ -4901,7 +4901,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 09/07/2026</t>
+          <t>Complete Holdings Dividend Summary - 09/14/2026</t>
         </is>
       </c>
     </row>
@@ -5005,7 +5005,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.00883876829813468</v>
+        <v>0.00946320755973527</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46255</v>
@@ -5058,7 +5058,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02305422717269788</v>
+        <v>0.02668498548328576</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46255</v>
@@ -5111,7 +5111,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.004986937847341924</v>
+        <v>0.005338793701200471</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5164,7 +5164,7 @@
         <v>2.184</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02466960386438792</v>
+        <v>0.0250789461211513</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46251</v>
@@ -5217,7 +5217,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03841005375174777</v>
+        <v>0.03957219387294963</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46251</v>
@@ -5270,7 +5270,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02533513789021478</v>
+        <v>0.02503037574256811</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46265</v>
@@ -5323,7 +5323,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.05372877854259377</v>
+        <v>0.05629362775477879</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46246</v>
@@ -5376,10 +5376,10 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.0184862591703806</v>
+        <v>0.0186580544393274</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>46182</v>
+        <v>46274</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>4.96</v>
@@ -5429,7 +5429,7 @@
         <v>0.96</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02419964820546709</v>
+        <v>0.02463433333150609</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46254</v>
@@ -5482,7 +5482,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.007251850465255884</v>
+        <v>0.007397361552028218</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46248</v>
@@ -5535,7 +5535,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01538461581456155</v>
+        <v>0.01520224384693243</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46209</v>
@@ -5588,7 +5588,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03413230964368608</v>
+        <v>0.03291115891894363</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46253</v>
@@ -5641,7 +5641,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.014506198907202</v>
+        <v>0.01446715458684541</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46211</v>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Dec</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="F18" s="7" t="n">
@@ -5694,7 +5694,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02663337418694604</v>
+        <v>0.02508574153301707</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46188</v>
@@ -5706,7 +5706,7 @@
         <v>46433</v>
       </c>
       <c r="L18" s="10" t="n">
-        <v>46368</v>
+        <v>46458</v>
       </c>
       <c r="M18" s="12" t="inlineStr">
         <is>
@@ -5747,7 +5747,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.04719763849938742</v>
+        <v>0.04971885038416789</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46188</v>
@@ -5800,7 +5800,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.0238650142641304</v>
+        <v>0.02491484184914842</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46247</v>
@@ -5853,7 +5853,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01769665194015332</v>
+        <v>0.01779070791836802</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5906,7 +5906,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>0.01515151568586133</v>
+        <v>0.01539665983034154</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>46223</v>
@@ -5959,7 +5959,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.02902974724923542</v>
+        <v>0.03000740561476674</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46268</v>
@@ -6012,7 +6012,7 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.01930542489909123</v>
+        <v>0.01974143087025879</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46262</v>
@@ -6065,7 +6065,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.05441039694455867</v>
+        <v>0.05595607625096392</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6118,7 +6118,7 @@
         <v>2</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>0.02637130929027715</v>
+        <v>0.02641310047223251</v>
       </c>
       <c r="I26" s="20" t="n">
         <v>46269</v>
@@ -6171,7 +6171,7 @@
         <v>3.28</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.03239186184874104</v>
+        <v>0.03249306950164277</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46204</v>
@@ -6224,7 +6224,7 @@
         <v>2.44</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.01473074142109956</v>
+        <v>0.01462479053918474</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46269</v>
@@ -6277,7 +6277,7 @@
         <v>5.36</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01947462044851735</v>
+        <v>0.01990567170011602</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46259</v>
@@ -6330,7 +6330,7 @@
         <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.01672986770838049</v>
+        <v>0.01699235314722998</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46209</v>
@@ -6383,7 +6383,7 @@
         <v>2.25</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.02008928571428572</v>
+        <v>0.0204202028393521</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46216</v>
@@ -6436,7 +6436,7 @@
         <v>3.16</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.01143105184521834</v>
+        <v>0.0127142515706196</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46203</v>
@@ -6489,7 +6489,7 @@
         <v>2.88</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03058298880746655</v>
+        <v>0.03080872803355954</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46199</v>
@@ -6542,7 +6542,7 @@
         <v>1.92</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.03686635815083875</v>
+        <v>0.03748535638894003</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46209</v>
@@ -6595,7 +6595,7 @@
         <v>3.64</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.007284370444425581</v>
+        <v>0.007252874320868801</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46254</v>
@@ -6607,7 +6607,7 @@
         <v>46278</v>
       </c>
       <c r="L35" s="10" t="n">
-        <v>46344</v>
+        <v>46709</v>
       </c>
       <c r="M35" s="12" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
         <v>3.48</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.02866320644948689</v>
+        <v>0.028948135474036</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46211</v>
@@ -6701,7 +6701,7 @@
         <v>1.64</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04270833163625671</v>
+        <v>0.04430037762617224</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46266</v>
@@ -6754,7 +6754,7 @@
         <v>1.158</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.02484978622141126</v>
+        <v>0.02673438847314084</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46251</v>
@@ -6807,7 +6807,7 @@
         <v>3.252</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.05309387755102041</v>
+        <v>0.05447236111291268</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46265</v>
@@ -6860,7 +6860,7 @@
         <v>4.76</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.03910935860492718</v>
+        <v>0.04061086969695727</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46231</v>
@@ -6913,10 +6913,10 @@
         <v>2.68</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.03636363786937607</v>
+        <v>0.03727399086403899</v>
       </c>
       <c r="I41" s="10" t="n">
-        <v>46182</v>
+        <v>46274</v>
       </c>
       <c r="J41" s="8" t="n">
         <v>0.06349206349206354</v>
@@ -6966,7 +6966,7 @@
         <v>5.92</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.0430138762622343</v>
+        <v>0.04294834704934376</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46269</v>
@@ -7019,7 +7019,7 @@
         <v>1.72</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.06045694038225009</v>
+        <v>0.0618816332174422</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46227</v>
@@ -7072,7 +7072,7 @@
         <v>3.36</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.02879670887223125</v>
+        <v>0.02863412689310154</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46268</v>
@@ -7125,7 +7125,7 @@
         <v>4.356</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.02974597055024585</v>
+        <v>0.02964170822323141</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46227</v>
@@ -7178,7 +7178,7 @@
         <v>2.204</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.04520098596940841</v>
+        <v>0.04570717428878286</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46198</v>
@@ -7231,7 +7231,7 @@
         <v>5.08</v>
       </c>
       <c r="H47" s="9" t="n">
-        <v>0.01991454025218246</v>
+        <v>0.01924971624665003</v>
       </c>
       <c r="I47" s="10" t="n">
         <v>46252</v>
@@ -7284,7 +7284,7 @@
         <v>3.92</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.01547755333783219</v>
+        <v>0.01568376395018629</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46252</v>
@@ -7337,7 +7337,7 @@
         <v>9.76</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.02548302872062663</v>
+        <v>0.02583787857341831</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46253</v>
@@ -7384,25 +7384,25 @@
         </is>
       </c>
       <c r="F50" s="7" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="G50" s="25" t="n">
-        <v>3.32</v>
+        <v>3.36</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.03410024629403103</v>
+        <v>0.03791041525582833</v>
       </c>
       <c r="I50" s="10" t="n">
-        <v>46181</v>
+        <v>46273</v>
       </c>
       <c r="J50" s="8" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.01204819277108435</v>
       </c>
       <c r="K50" s="10" t="n">
-        <v>46592</v>
+        <v>46591</v>
       </c>
       <c r="L50" s="10" t="n">
-        <v>46632</v>
+        <v>46633</v>
       </c>
       <c r="M50" s="12" t="inlineStr">
         <is>
@@ -7443,7 +7443,7 @@
         <v>5.2</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.04736746272382592</v>
+        <v>0.04881483149978388</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46188</v>
@@ -7496,7 +7496,7 @@
         <v>3.896</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.04397787742467318</v>
+        <v>0.04231333292565891</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46112</v>
@@ -7549,7 +7549,7 @@
         <v>5.68</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.0219780217704021</v>
+        <v>0.02153962736846832</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46234</v>
@@ -7602,7 +7602,7 @@
         <v>2.124</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.03308411372219163</v>
+        <v>0.03364219619018467</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46241</v>
@@ -7655,7 +7655,7 @@
         <v>5.68</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.01961190558580643</v>
+        <v>0.0199424192610679</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46265</v>
@@ -7708,7 +7708,7 @@
         <v>2.832</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.05648185150526099</v>
+        <v>0.05532352119915055</v>
       </c>
       <c r="I56" s="10" t="n">
         <v>46213</v>
@@ -7761,7 +7761,7 @@
         <v>4.12</v>
       </c>
       <c r="H57" s="9" t="n">
-        <v>0.02583558016217738</v>
+        <v>0.02451651249736115</v>
       </c>
       <c r="I57" s="10" t="n">
         <v>46251</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-10-05
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 09/28/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 10/05/2026</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-245</v>
+        <v>-252</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06040386222854276</v>
+        <v>0.06260236491789237</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         <v>46305</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="J7" s="10" t="n">
         <v>46339</v>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.02871523995292049</v>
+        <v>0.0269120722736316</v>
       </c>
     </row>
     <row r="8">
@@ -772,8 +772,8 @@
       <c r="H8" s="10" t="n">
         <v>46311</v>
       </c>
-      <c r="I8" s="14" t="n">
-        <v>18</v>
+      <c r="I8" s="13" t="n">
+        <v>11</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46386</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.01157763600694031</v>
+        <v>0.0116302613355222</v>
       </c>
     </row>
     <row r="9">
@@ -819,7 +819,7 @@
         <v>46318</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46352</v>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.02119327413458831</v>
+        <v>0.02049834685596653</v>
       </c>
     </row>
     <row r="10">
@@ -865,7 +865,7 @@
         <v>46322</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46338</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.02619193836660545</v>
+        <v>0.02542835780877885</v>
       </c>
     </row>
     <row r="11">
@@ -911,7 +911,7 @@
         <v>46329</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46338</v>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.00785828876337411</v>
+        <v>0.007742684745454336</v>
       </c>
     </row>
     <row r="12">
@@ -957,7 +957,7 @@
         <v>46332</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46346</v>
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.02629593680273037</v>
+        <v>0.02675878779765391</v>
       </c>
     </row>
     <row r="13">
@@ -1003,7 +1003,7 @@
         <v>46341</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46340</v>
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.02525206111259398</v>
+        <v>0.025221915188599</v>
       </c>
     </row>
     <row r="14">
@@ -1049,7 +1049,7 @@
         <v>46344</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46385</v>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.03987953020551666</v>
+        <v>0.04340945104841216</v>
       </c>
     </row>
     <row r="15">
@@ -1095,7 +1095,7 @@
         <v>46347</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46358</v>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.04558087884561619</v>
+        <v>0.0497045022909573</v>
       </c>
     </row>
     <row r="16">
@@ -1141,7 +1141,7 @@
         <v>46352</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46400</v>
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.05962859115015496</v>
+        <v>0.05796241542035767</v>
       </c>
     </row>
     <row r="17">
@@ -1187,7 +1187,7 @@
         <v>46360</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46371</v>
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.05089367117307898</v>
+        <v>0.05169230769230769</v>
       </c>
     </row>
     <row r="18">
@@ -1233,7 +1233,7 @@
         <v>46366</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46432</v>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.02434900172108285</v>
+        <v>0.0250733801190597</v>
       </c>
     </row>
     <row r="19">
@@ -1279,7 +1279,7 @@
         <v>46380</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46436</v>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.026044492243725</v>
+        <v>0.02546081297917674</v>
       </c>
     </row>
     <row r="20">
@@ -1325,7 +1325,7 @@
         <v>46383</v>
       </c>
       <c r="I20" s="21" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="J20" s="20" t="n">
         <v>46404</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="L20" s="19" t="n">
-        <v>0.01510303393679408</v>
+        <v>0.0152012882447665</v>
       </c>
     </row>
     <row r="21">
@@ -1371,7 +1371,7 @@
         <v>46402</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46483</v>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.01466044423432771</v>
+        <v>0.01482915257546235</v>
       </c>
     </row>
     <row r="22">
@@ -1417,7 +1417,7 @@
         <v>46411</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46435</v>
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.04049539028131194</v>
+        <v>0.03974558303886926</v>
       </c>
     </row>
     <row r="23">
@@ -1463,7 +1463,7 @@
         <v>46417</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46433</v>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.03436293486905094</v>
+        <v>0.03491993354817895</v>
       </c>
     </row>
     <row r="24">
@@ -1509,7 +1509,7 @@
         <v>46423</v>
       </c>
       <c r="I24" s="14" t="n">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46473</v>
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.03028242544905738</v>
+        <v>0.03123398452246422</v>
       </c>
     </row>
     <row r="25">
@@ -1555,7 +1555,7 @@
         <v>46428</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46452</v>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01661898840947346</v>
+        <v>0.01707069676200025</v>
       </c>
     </row>
     <row r="26">
@@ -1601,7 +1601,7 @@
         <v>46428</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46460</v>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.04955920751734383</v>
+        <v>0.05039736368113923</v>
       </c>
     </row>
     <row r="27">
@@ -1647,7 +1647,7 @@
         <v>46429</v>
       </c>
       <c r="I27" s="21" t="n">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J27" s="20" t="n">
         <v>46450</v>
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="L27" s="19" t="n">
-        <v>0.02734481838515112</v>
+        <v>0.0275824016146412</v>
       </c>
     </row>
     <row r="28">
@@ -1693,7 +1693,7 @@
         <v>46431</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46480</v>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.01573991652591106</v>
+        <v>0.01496259367888212</v>
       </c>
     </row>
     <row r="29">
@@ -1739,7 +1739,7 @@
         <v>46432</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46455</v>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.04014379739729774</v>
+        <v>0.03948725344843111</v>
       </c>
     </row>
     <row r="30">
@@ -1785,7 +1785,7 @@
         <v>46433</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46425</v>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.004863235712254763</v>
+        <v>0.004618563878007072</v>
       </c>
     </row>
     <row r="31">
@@ -1831,7 +1831,7 @@
         <v>46433</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46383</v>
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.01946180602749289</v>
+        <v>0.01960488686266767</v>
       </c>
     </row>
     <row r="32">
@@ -1877,7 +1877,7 @@
         <v>46433</v>
       </c>
       <c r="I32" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46458</v>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.02705845030636119</v>
+        <v>0.02692469447517261</v>
       </c>
     </row>
     <row r="33">
@@ -1923,7 +1923,7 @@
         <v>46433</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46634</v>
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.0289443082784107</v>
+        <v>0.02993185232025556</v>
       </c>
     </row>
     <row r="34">
@@ -1969,7 +1969,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46608</v>
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.03422494284562026</v>
+        <v>0.03558086960144769</v>
       </c>
     </row>
     <row r="35">
@@ -2015,7 +2015,7 @@
         <v>46440</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46450</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.01017633144783744</v>
+        <v>0.01000906021484749</v>
       </c>
     </row>
     <row r="36">
@@ -2061,7 +2061,7 @@
         <v>46441</v>
       </c>
       <c r="I36" s="14" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46456</v>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.03197583639308245</v>
+        <v>0.03327086122266845</v>
       </c>
     </row>
     <row r="37">
@@ -2107,7 +2107,7 @@
         <v>46452</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46487</v>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.018949438093953</v>
+        <v>0.01926572184075763</v>
       </c>
     </row>
     <row r="38">
@@ -2153,7 +2153,7 @@
         <v>46461</v>
       </c>
       <c r="I38" s="14" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46665</v>
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.01768920061562391</v>
+        <v>0.01813072291056532</v>
       </c>
     </row>
     <row r="39">
@@ -2184,13 +2184,13 @@
         </is>
       </c>
       <c r="D39" s="7" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="E39" s="7" t="n">
         <v>0.271</v>
       </c>
-      <c r="E39" s="7" t="n">
-        <v>0.27</v>
-      </c>
       <c r="F39" s="8" t="n">
-        <v>0.003703703703703707</v>
+        <v>0.003690036900369007</v>
       </c>
       <c r="G39" s="9" t="n">
         <v>0.02</v>
@@ -2199,7 +2199,7 @@
         <v>46461</v>
       </c>
       <c r="I39" s="14" t="n">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46386</v>
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.05867388443418352</v>
+        <v>0.06097515550966866</v>
       </c>
     </row>
     <row r="40">
@@ -2245,7 +2245,7 @@
         <v>46488</v>
       </c>
       <c r="I40" s="14" t="n">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46498</v>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.02960948806953896</v>
+        <v>0.03003827202933425</v>
       </c>
     </row>
     <row r="41">
@@ -2291,7 +2291,7 @@
         <v>46492</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46501</v>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.02055733268831431</v>
+        <v>0.02102116058315701</v>
       </c>
     </row>
     <row r="42">
@@ -2322,13 +2322,13 @@
         </is>
       </c>
       <c r="D42" s="7" t="n">
+        <v>1.021</v>
+      </c>
+      <c r="E42" s="7" t="n">
         <v>0.974</v>
       </c>
-      <c r="E42" s="7" t="n">
-        <v>0.994</v>
-      </c>
       <c r="F42" s="8" t="n">
-        <v>0.001006036217303824</v>
+        <v>0.04825462012320322</v>
       </c>
       <c r="G42" s="9" t="n">
         <v>0.02</v>
@@ -2337,7 +2337,7 @@
         <v>46492</v>
       </c>
       <c r="I42" s="14" t="n">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46376</v>
@@ -2348,7 +2348,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.04263981485045694</v>
+        <v>0.04847765287972164</v>
       </c>
     </row>
     <row r="43">
@@ -2383,7 +2383,7 @@
         <v>46493</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46531</v>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.01969936444610691</v>
+        <v>0.02101466341764813</v>
       </c>
     </row>
     <row r="44">
@@ -2429,7 +2429,7 @@
         <v>46504</v>
       </c>
       <c r="I44" s="14" t="n">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46562</v>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.04796517874658265</v>
+        <v>0.04941704204942651</v>
       </c>
     </row>
     <row r="45">
@@ -2473,7 +2473,7 @@
         <v>46505</v>
       </c>
       <c r="I45" s="21" t="n">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="J45" s="20" t="n">
         <v>46526</v>
@@ -2484,7 +2484,7 @@
         </is>
       </c>
       <c r="L45" s="19" t="n">
-        <v>0.01969831987068282</v>
+        <v>0.01903762580466897</v>
       </c>
     </row>
     <row r="46">
@@ -2519,7 +2519,7 @@
         <v>46508</v>
       </c>
       <c r="I46" s="14" t="n">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46518</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.04749076963560451</v>
+        <v>0.04781997143077665</v>
       </c>
     </row>
     <row r="47">
@@ -2565,7 +2565,7 @@
         <v>46515</v>
       </c>
       <c r="I47" s="14" t="n">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46542</v>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.04644933337595475</v>
+        <v>0.04754065390450687</v>
       </c>
     </row>
     <row r="48">
@@ -2611,7 +2611,7 @@
         <v>46532</v>
       </c>
       <c r="I48" s="14" t="n">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46563</v>
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.03276637021439819</v>
+        <v>0.03316635032377153</v>
       </c>
     </row>
     <row r="49">
@@ -2657,7 +2657,7 @@
         <v>46589</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46629</v>
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.02066506695303406</v>
+        <v>0.02059799423192274</v>
       </c>
     </row>
     <row r="50">
@@ -2703,7 +2703,7 @@
         <v>46591</v>
       </c>
       <c r="I50" s="14" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46633</v>
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.03726707923163132</v>
+        <v>0.0376935160759064</v>
       </c>
     </row>
     <row r="51">
@@ -2749,7 +2749,7 @@
         <v>46594</v>
       </c>
       <c r="I51" s="14" t="n">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46613</v>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.01576354660457816</v>
+        <v>0.01569066954036555</v>
       </c>
     </row>
     <row r="52">
@@ -2795,7 +2795,7 @@
         <v>46595</v>
       </c>
       <c r="I52" s="14" t="n">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46614</v>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.0264903876291373</v>
+        <v>0.02679754601226994</v>
       </c>
     </row>
     <row r="53">
@@ -2841,7 +2841,7 @@
         <v>46597</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46611</v>
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.06110975334452722</v>
+        <v>0.0615498241205511</v>
       </c>
     </row>
     <row r="54">
@@ -2887,7 +2887,7 @@
         <v>46598</v>
       </c>
       <c r="I54" s="14" t="n">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46629</v>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.02627132204797521</v>
+        <v>0.02686576971590722</v>
       </c>
     </row>
     <row r="55">
@@ -2918,22 +2918,22 @@
         </is>
       </c>
       <c r="D55" s="7" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="E55" s="7" t="n">
         <v>0.82</v>
       </c>
-      <c r="E55" s="7" t="n">
-        <v>0.8</v>
-      </c>
       <c r="F55" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="G55" s="9" t="n">
         <v>0.04</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>46628</v>
+        <v>46614</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>335</v>
+        <v>314</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46662</v>
@@ -2944,7 +2944,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.03395269278011557</v>
+        <v>0.03503772989535116</v>
       </c>
     </row>
     <row r="56">
@@ -2979,7 +2979,7 @@
         <v>46643</v>
       </c>
       <c r="I56" s="14" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46709</v>
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.007144434529232485</v>
+        <v>0.006893939393939394</v>
       </c>
     </row>
     <row r="57">
@@ -3025,7 +3025,7 @@
         <v>46645</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46668</v>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.06022328353230328</v>
+        <v>0.06189487343217447</v>
       </c>
     </row>
     <row r="58">
@@ -3071,7 +3071,7 @@
         <v>46650</v>
       </c>
       <c r="I58" s="14" t="n">
-        <v>357</v>
+        <v>350</v>
       </c>
       <c r="J58" s="10" t="n">
         <v>46690</v>
@@ -3082,7 +3082,7 @@
         </is>
       </c>
       <c r="L58" s="9" t="n">
-        <v>0.0205462099807986</v>
+        <v>0.0196041137387245</v>
       </c>
     </row>
   </sheetData>
@@ -3117,7 +3117,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 09/28/2026</t>
+          <t>Expected Increase Announcements by Month - 10/05/2026</t>
         </is>
       </c>
     </row>
@@ -4199,10 +4199,10 @@
         <v>46386</v>
       </c>
       <c r="D57" s="7" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>0.003703703703703707</v>
+        <v>0.003690036900369007</v>
       </c>
       <c r="F57" s="12" t="inlineStr">
         <is>
@@ -4310,10 +4310,10 @@
         <v>46376</v>
       </c>
       <c r="D63" s="7" t="n">
-        <v>0.974</v>
+        <v>1.021</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>0.001006036217303824</v>
+        <v>0.04825462012320322</v>
       </c>
       <c r="F63" s="12" t="inlineStr">
         <is>
@@ -4733,16 +4733,16 @@
         </is>
       </c>
       <c r="B85" s="10" t="n">
-        <v>46628</v>
+        <v>46614</v>
       </c>
       <c r="C85" s="10" t="n">
         <v>46662</v>
       </c>
       <c r="D85" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="E85" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="F85" s="12" t="inlineStr">
         <is>
@@ -4900,7 +4900,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 09/28/2026</t>
+          <t>Complete Holdings Dividend Summary - 10/05/2026</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01017633144783744</v>
+        <v>0.01000906021484749</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46255</v>
@@ -5057,7 +5057,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.02434900172108285</v>
+        <v>0.0250733801190597</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46255</v>
@@ -5110,7 +5110,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.004863235712254763</v>
+        <v>0.004618563878007072</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5163,7 +5163,7 @@
         <v>2.184</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.0264903876291373</v>
+        <v>0.02679754601226994</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46251</v>
@@ -5216,7 +5216,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.04049539028131194</v>
+        <v>0.03974558303886926</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46251</v>
@@ -5269,7 +5269,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02627132204797521</v>
+        <v>0.02686576971590722</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46265</v>
@@ -5322,7 +5322,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.06110975334452722</v>
+        <v>0.0615498241205511</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46246</v>
@@ -5375,7 +5375,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.01946180602749289</v>
+        <v>0.01960488686266767</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46274</v>
@@ -5428,7 +5428,7 @@
         <v>0.96</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.026044492243725</v>
+        <v>0.02546081297917674</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46254</v>
@@ -5481,7 +5481,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.00785828876337411</v>
+        <v>0.007742684745454336</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46248</v>
@@ -5534,10 +5534,10 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01573991652591106</v>
+        <v>0.01496259367888212</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>46209</v>
+        <v>46297</v>
       </c>
       <c r="J15" s="8" t="n">
         <v>0.02439024390243905</v>
@@ -5587,7 +5587,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03436293486905094</v>
+        <v>0.03491993354817895</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46253</v>
@@ -5640,7 +5640,7 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01466044423432771</v>
+        <v>0.01482915257546235</v>
       </c>
       <c r="I17" s="10" t="n">
         <v>46211</v>
@@ -5693,7 +5693,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02705845030636119</v>
+        <v>0.02692469447517261</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46280</v>
@@ -5746,7 +5746,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.05089367117307898</v>
+        <v>0.05169230769230769</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46280</v>
@@ -5799,7 +5799,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02619193836660545</v>
+        <v>0.02542835780877885</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46247</v>
@@ -5852,7 +5852,7 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.018949438093953</v>
+        <v>0.01926572184075763</v>
       </c>
       <c r="I21" s="10" t="n">
         <v>46205</v>
@@ -5905,7 +5905,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>0.01510303393679408</v>
+        <v>0.0152012882447665</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>46223</v>
@@ -5958,7 +5958,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.03197583639308245</v>
+        <v>0.03327086122266845</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46268</v>
@@ -6011,7 +6011,7 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.02119327413458831</v>
+        <v>0.02049834685596653</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46262</v>
@@ -6064,7 +6064,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.05962859115015496</v>
+        <v>0.05796241542035767</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6117,7 +6117,7 @@
         <v>2</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>0.02734481838515112</v>
+        <v>0.0275824016146412</v>
       </c>
       <c r="I26" s="20" t="n">
         <v>46269</v>
@@ -6164,22 +6164,22 @@
         </is>
       </c>
       <c r="F27" s="7" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="G27" s="26" t="n">
-        <v>3.28</v>
+        <v>3.32</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.03395269278011557</v>
+        <v>0.03503772989535116</v>
       </c>
       <c r="I27" s="10" t="n">
-        <v>46204</v>
+        <v>46296</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>0.02499999999999988</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="K27" s="10" t="n">
-        <v>46628</v>
+        <v>46614</v>
       </c>
       <c r="L27" s="10" t="n">
         <v>46662</v>
@@ -6223,7 +6223,7 @@
         <v>2.44</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.01661898840947346</v>
+        <v>0.01707069676200025</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46269</v>
@@ -6276,7 +6276,7 @@
         <v>5.36</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01969936444610691</v>
+        <v>0.02101466341764813</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46259</v>
@@ -6329,7 +6329,7 @@
         <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.01768920061562391</v>
+        <v>0.01813072291056532</v>
       </c>
       <c r="I30" s="10" t="n">
         <v>46209</v>
@@ -6382,7 +6382,7 @@
         <v>2.25</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.02055733268831431</v>
+        <v>0.02102116058315701</v>
       </c>
       <c r="I31" s="10" t="n">
         <v>46216</v>
@@ -6435,10 +6435,10 @@
         <v>3.16</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.01157763600694031</v>
+        <v>0.0116302613355222</v>
       </c>
       <c r="I32" s="10" t="n">
-        <v>46203</v>
+        <v>46295</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>0.05333333333333338</v>
@@ -6488,7 +6488,7 @@
         <v>2.88</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03276637021439819</v>
+        <v>0.03316635032377153</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46290</v>
@@ -6541,7 +6541,7 @@
         <v>1.92</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.03987953020551666</v>
+        <v>0.04340945104841216</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46209</v>
@@ -6594,7 +6594,7 @@
         <v>3.64</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.007144434529232485</v>
+        <v>0.006893939393939394</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46254</v>
@@ -6647,7 +6647,7 @@
         <v>3.48</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.02871523995292049</v>
+        <v>0.0269120722736316</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46211</v>
@@ -6700,7 +6700,7 @@
         <v>1.64</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.04558087884561619</v>
+        <v>0.0497045022909573</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46266</v>
@@ -6753,7 +6753,7 @@
         <v>1.158</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03028242544905738</v>
+        <v>0.03123398452246422</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46251</v>
@@ -6800,19 +6800,19 @@
         </is>
       </c>
       <c r="F39" s="7" t="n">
-        <v>0.271</v>
+        <v>0.272</v>
       </c>
       <c r="G39" s="26" t="n">
-        <v>3.252</v>
+        <v>3.264</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.05867388443418352</v>
+        <v>0.06097515550966866</v>
       </c>
       <c r="I39" s="10" t="n">
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>0.003703703703703707</v>
+        <v>0.003690036900369007</v>
       </c>
       <c r="K39" s="10" t="n">
         <v>46461</v>
@@ -6859,7 +6859,7 @@
         <v>4.76</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.04749076963560451</v>
+        <v>0.04781997143077665</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46231</v>
@@ -6912,7 +6912,7 @@
         <v>2.68</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.04014379739729774</v>
+        <v>0.03948725344843111</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46274</v>
@@ -6965,7 +6965,7 @@
         <v>5.92</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.04644933337595475</v>
+        <v>0.04754065390450687</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46269</v>
@@ -7018,7 +7018,7 @@
         <v>1.72</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.06040386222854276</v>
+        <v>0.06260236491789237</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46227</v>
@@ -7071,7 +7071,7 @@
         <v>3.36</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.0289443082784107</v>
+        <v>0.02993185232025556</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46268</v>
@@ -7124,7 +7124,7 @@
         <v>4.356</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.02960948806953896</v>
+        <v>0.03003827202933425</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46227</v>
@@ -7177,7 +7177,7 @@
         <v>2.204</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.04796517874658265</v>
+        <v>0.04941704204942651</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46290</v>
@@ -7230,7 +7230,7 @@
         <v>5.08</v>
       </c>
       <c r="H47" s="19" t="n">
-        <v>0.01969831987068282</v>
+        <v>0.01903762580466897</v>
       </c>
       <c r="I47" s="20" t="n">
         <v>46252</v>
@@ -7283,7 +7283,7 @@
         <v>3.92</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.01576354660457816</v>
+        <v>0.01569066954036555</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46252</v>
@@ -7336,7 +7336,7 @@
         <v>9.76</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.02629593680273037</v>
+        <v>0.02675878779765391</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46253</v>
@@ -7389,7 +7389,7 @@
         <v>3.36</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.03726707923163132</v>
+        <v>0.0376935160759064</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46273</v>
@@ -7442,7 +7442,7 @@
         <v>5.2</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.04955920751734383</v>
+        <v>0.05039736368113923</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46280</v>
@@ -7489,19 +7489,19 @@
         </is>
       </c>
       <c r="F52" s="7" t="n">
-        <v>0.974</v>
+        <v>1.021</v>
       </c>
       <c r="G52" s="26" t="n">
-        <v>3.896</v>
+        <v>4.084</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.04263981485045694</v>
+        <v>0.04847765287972164</v>
       </c>
       <c r="I52" s="10" t="n">
-        <v>46112</v>
+        <v>46295</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>0.001006036217303824</v>
+        <v>0.04825462012320322</v>
       </c>
       <c r="K52" s="10" t="n">
         <v>46492</v>
@@ -7548,7 +7548,7 @@
         <v>5.68</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.0205462099807986</v>
+        <v>0.0196041137387245</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46234</v>
@@ -7601,7 +7601,7 @@
         <v>2.124</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.03422494284562026</v>
+        <v>0.03558086960144769</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46241</v>
@@ -7654,7 +7654,7 @@
         <v>5.68</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.02066506695303406</v>
+        <v>0.02059799423192274</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46265</v>
@@ -7707,7 +7707,7 @@
         <v>2.832</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.06022328353230328</v>
+        <v>0.06189487343217447</v>
       </c>
       <c r="I56" s="10" t="n">
         <v>46213</v>
@@ -7760,7 +7760,7 @@
         <v>4.12</v>
       </c>
       <c r="H57" s="9" t="n">
-        <v>0.02525206111259398</v>
+        <v>0.025221915188599</v>
       </c>
       <c r="I57" s="10" t="n">
         <v>46251</v>

</xml_diff>

<commit_message>
Update dividend calendar 2026-10-12
</commit_message>
<xml_diff>
--- a/data/dividend_calendar.xlsx
+++ b/data/dividend_calendar.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estimated Dividend Calendar: Anticipated Announcements - 10/05/2026</t>
+          <t>Estimated Dividend Calendar: Anticipated Announcements - 10/12/2026</t>
         </is>
       </c>
     </row>
@@ -681,7 +681,7 @@
         <v>46048</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>-252</v>
+        <v>-259</v>
       </c>
       <c r="J6" s="10" t="n">
         <v>46413</v>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="L6" s="9" t="n">
-        <v>0.06260236491789237</v>
+        <v>0.060584714229587</v>
       </c>
     </row>
     <row r="7">
@@ -726,11 +726,11 @@
       <c r="H7" s="10" t="n">
         <v>46305</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <v>5</v>
+      <c r="I7" s="11" t="n">
+        <v>-2</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>46339</v>
+        <v>46704</v>
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.0269120722736316</v>
+        <v>0.02696629149713606</v>
       </c>
     </row>
     <row r="8">
@@ -773,7 +773,7 @@
         <v>46311</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>46386</v>
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="L8" s="9" t="n">
-        <v>0.0116302613355222</v>
+        <v>0.01212074758762932</v>
       </c>
     </row>
     <row r="9">
@@ -818,8 +818,8 @@
       <c r="H9" s="10" t="n">
         <v>46318</v>
       </c>
-      <c r="I9" s="14" t="n">
-        <v>18</v>
+      <c r="I9" s="13" t="n">
+        <v>11</v>
       </c>
       <c r="J9" s="10" t="n">
         <v>46352</v>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="L9" s="9" t="n">
-        <v>0.02049834685596653</v>
+        <v>0.02065597808138082</v>
       </c>
     </row>
     <row r="10">
@@ -865,7 +865,7 @@
         <v>46322</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="J10" s="10" t="n">
         <v>46338</v>
@@ -876,7 +876,7 @@
         </is>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0.02542835780877885</v>
+        <v>0.02477139648518534</v>
       </c>
     </row>
     <row r="11">
@@ -911,7 +911,7 @@
         <v>46329</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J11" s="10" t="n">
         <v>46338</v>
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="L11" s="9" t="n">
-        <v>0.007742684745454336</v>
+        <v>0.007395538275760539</v>
       </c>
     </row>
     <row r="12">
@@ -957,7 +957,7 @@
         <v>46332</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="J12" s="10" t="n">
         <v>46346</v>
@@ -968,7 +968,7 @@
         </is>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0.02675878779765391</v>
+        <v>0.0270262782600054</v>
       </c>
     </row>
     <row r="13">
@@ -1003,7 +1003,7 @@
         <v>46341</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>46340</v>
@@ -1014,7 +1014,7 @@
         </is>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0.025221915188599</v>
+        <v>0.02392427756445954</v>
       </c>
     </row>
     <row r="14">
@@ -1049,7 +1049,7 @@
         <v>46344</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>46385</v>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0.04340945104841216</v>
+        <v>0.04253433819142445</v>
       </c>
     </row>
     <row r="15">
@@ -1095,7 +1095,7 @@
         <v>46347</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J15" s="10" t="n">
         <v>46358</v>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="L15" s="9" t="n">
-        <v>0.0497045022909573</v>
+        <v>0.04726905935798738</v>
       </c>
     </row>
     <row r="16">
@@ -1141,7 +1141,7 @@
         <v>46352</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="J16" s="10" t="n">
         <v>46400</v>
@@ -1152,7 +1152,7 @@
         </is>
       </c>
       <c r="L16" s="9" t="n">
-        <v>0.05796241542035767</v>
+        <v>0.06113719328824217</v>
       </c>
     </row>
     <row r="17">
@@ -1181,13 +1181,13 @@
         <v>0.01204819277108435</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="H17" s="10" t="n">
         <v>46360</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="J17" s="10" t="n">
         <v>46371</v>
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0.05169230769230769</v>
+        <v>0.05388501362627859</v>
       </c>
     </row>
     <row r="18">
@@ -1233,7 +1233,7 @@
         <v>46366</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="J18" s="10" t="n">
         <v>46432</v>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0.0250733801190597</v>
+        <v>0.02435106070044935</v>
       </c>
     </row>
     <row r="19">
@@ -1279,7 +1279,7 @@
         <v>46380</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="J19" s="10" t="n">
         <v>46436</v>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0.02546081297917674</v>
+        <v>0.02474864597427012</v>
       </c>
     </row>
     <row r="20">
@@ -1325,7 +1325,7 @@
         <v>46383</v>
       </c>
       <c r="I20" s="21" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="J20" s="20" t="n">
         <v>46404</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="L20" s="19" t="n">
-        <v>0.0152012882447665</v>
+        <v>0.01507024206908392</v>
       </c>
     </row>
     <row r="21">
@@ -1371,7 +1371,7 @@
         <v>46402</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J21" s="10" t="n">
         <v>46483</v>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="L21" s="9" t="n">
-        <v>0.01482915257546235</v>
+        <v>0.01480142827673315</v>
       </c>
     </row>
     <row r="22">
@@ -1417,7 +1417,7 @@
         <v>46411</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="J22" s="10" t="n">
         <v>46435</v>
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="L22" s="9" t="n">
-        <v>0.03974558303886926</v>
+        <v>0.0369854010936235</v>
       </c>
     </row>
     <row r="23">
@@ -1463,7 +1463,7 @@
         <v>46417</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="J23" s="10" t="n">
         <v>46433</v>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0.03491993354817895</v>
+        <v>0.03298357685968453</v>
       </c>
     </row>
     <row r="24">
@@ -1509,7 +1509,7 @@
         <v>46423</v>
       </c>
       <c r="I24" s="14" t="n">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J24" s="10" t="n">
         <v>46473</v>
@@ -1520,7 +1520,7 @@
         </is>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0.03123398452246422</v>
+        <v>0.03014055323240503</v>
       </c>
     </row>
     <row r="25">
@@ -1555,7 +1555,7 @@
         <v>46428</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="J25" s="10" t="n">
         <v>46452</v>
@@ -1566,7 +1566,7 @@
         </is>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0.01707069676200025</v>
+        <v>0.01631015976237089</v>
       </c>
     </row>
     <row r="26">
@@ -1601,7 +1601,7 @@
         <v>46428</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="J26" s="10" t="n">
         <v>46460</v>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="L26" s="9" t="n">
-        <v>0.05039736368113923</v>
+        <v>0.05061812352845635</v>
       </c>
     </row>
     <row r="27">
@@ -1647,7 +1647,7 @@
         <v>46429</v>
       </c>
       <c r="I27" s="21" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="J27" s="20" t="n">
         <v>46450</v>
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="L27" s="19" t="n">
-        <v>0.0275824016146412</v>
+        <v>0.02748952065840456</v>
       </c>
     </row>
     <row r="28">
@@ -1693,7 +1693,7 @@
         <v>46431</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="J28" s="10" t="n">
         <v>46480</v>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="L28" s="9" t="n">
-        <v>0.01496259367888212</v>
+        <v>0.01454306253370746</v>
       </c>
     </row>
     <row r="29">
@@ -1739,7 +1739,7 @@
         <v>46432</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="J29" s="10" t="n">
         <v>46455</v>
@@ -1750,7 +1750,7 @@
         </is>
       </c>
       <c r="L29" s="9" t="n">
-        <v>0.03948725344843111</v>
+        <v>0.03777308125827056</v>
       </c>
     </row>
     <row r="30">
@@ -1785,7 +1785,7 @@
         <v>46433</v>
       </c>
       <c r="I30" s="14" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="J30" s="10" t="n">
         <v>46425</v>
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="L30" s="9" t="n">
-        <v>0.004618563878007072</v>
+        <v>0.004833085693226959</v>
       </c>
     </row>
     <row r="31">
@@ -1831,7 +1831,7 @@
         <v>46433</v>
       </c>
       <c r="I31" s="14" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="J31" s="10" t="n">
         <v>46383</v>
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="L31" s="9" t="n">
-        <v>0.01960488686266767</v>
+        <v>0.01841164230021915</v>
       </c>
     </row>
     <row r="32">
@@ -1877,7 +1877,7 @@
         <v>46433</v>
       </c>
       <c r="I32" s="14" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="J32" s="10" t="n">
         <v>46458</v>
@@ -1888,7 +1888,7 @@
         </is>
       </c>
       <c r="L32" s="9" t="n">
-        <v>0.02692469447517261</v>
+        <v>0.02608518459263433</v>
       </c>
     </row>
     <row r="33">
@@ -1923,7 +1923,7 @@
         <v>46433</v>
       </c>
       <c r="I33" s="14" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="J33" s="10" t="n">
         <v>46634</v>
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="L33" s="9" t="n">
-        <v>0.02993185232025556</v>
+        <v>0.03130677936678974</v>
       </c>
     </row>
     <row r="34">
@@ -1969,7 +1969,7 @@
         <v>46433</v>
       </c>
       <c r="I34" s="14" t="n">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="J34" s="10" t="n">
         <v>46608</v>
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="L34" s="9" t="n">
-        <v>0.03558086960144769</v>
+        <v>0.03395140590432928</v>
       </c>
     </row>
     <row r="35">
@@ -2015,7 +2015,7 @@
         <v>46440</v>
       </c>
       <c r="I35" s="14" t="n">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="J35" s="10" t="n">
         <v>46450</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="L35" s="9" t="n">
-        <v>0.01000906021484749</v>
+        <v>0.01032212162618396</v>
       </c>
     </row>
     <row r="36">
@@ -2061,7 +2061,7 @@
         <v>46441</v>
       </c>
       <c r="I36" s="14" t="n">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="J36" s="10" t="n">
         <v>46456</v>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="L36" s="9" t="n">
-        <v>0.03327086122266845</v>
+        <v>0.03219121426382717</v>
       </c>
     </row>
     <row r="37">
@@ -2107,7 +2107,7 @@
         <v>46452</v>
       </c>
       <c r="I37" s="14" t="n">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="J37" s="10" t="n">
         <v>46487</v>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="L37" s="9" t="n">
-        <v>0.01926572184075763</v>
+        <v>0.01906817724130214</v>
       </c>
     </row>
     <row r="38">
@@ -2138,13 +2138,13 @@
         </is>
       </c>
       <c r="D38" s="7" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E38" s="7" t="n">
         <v>1.5</v>
       </c>
-      <c r="E38" s="7" t="n">
-        <v>1.4</v>
-      </c>
       <c r="F38" s="8" t="n">
-        <v>0.07142857142857149</v>
+        <v>0.09999999999999994</v>
       </c>
       <c r="G38" s="9" t="n">
         <v>0.06</v>
@@ -2153,7 +2153,7 @@
         <v>46461</v>
       </c>
       <c r="I38" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J38" s="10" t="n">
         <v>46665</v>
@@ -2164,7 +2164,7 @@
         </is>
       </c>
       <c r="L38" s="9" t="n">
-        <v>0.01813072291056532</v>
+        <v>0.01974688024131375</v>
       </c>
     </row>
     <row r="39">
@@ -2199,7 +2199,7 @@
         <v>46461</v>
       </c>
       <c r="I39" s="14" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J39" s="10" t="n">
         <v>46386</v>
@@ -2210,7 +2210,7 @@
         </is>
       </c>
       <c r="L39" s="9" t="n">
-        <v>0.06097515550966866</v>
+        <v>0.06026977174155138</v>
       </c>
     </row>
     <row r="40">
@@ -2245,7 +2245,7 @@
         <v>46488</v>
       </c>
       <c r="I40" s="14" t="n">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="J40" s="10" t="n">
         <v>46498</v>
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="L40" s="9" t="n">
-        <v>0.03003827202933425</v>
+        <v>0.02866072298257646</v>
       </c>
     </row>
     <row r="41">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="D41" s="7" t="n">
-        <v>1.125</v>
+        <v>1.084</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>1.087</v>
@@ -2291,7 +2291,7 @@
         <v>46492</v>
       </c>
       <c r="I41" s="14" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="J41" s="10" t="n">
         <v>46501</v>
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="L41" s="9" t="n">
-        <v>0.02102116058315701</v>
+        <v>0.01961369636922693</v>
       </c>
     </row>
     <row r="42">
@@ -2337,7 +2337,7 @@
         <v>46492</v>
       </c>
       <c r="I42" s="14" t="n">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="J42" s="10" t="n">
         <v>46376</v>
@@ -2348,7 +2348,7 @@
         </is>
       </c>
       <c r="L42" s="9" t="n">
-        <v>0.04847765287972164</v>
+        <v>0.04612083409655995</v>
       </c>
     </row>
     <row r="43">
@@ -2383,7 +2383,7 @@
         <v>46493</v>
       </c>
       <c r="I43" s="14" t="n">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J43" s="10" t="n">
         <v>46531</v>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="L43" s="9" t="n">
-        <v>0.02101466341764813</v>
+        <v>0.02043461780192916</v>
       </c>
     </row>
     <row r="44">
@@ -2429,7 +2429,7 @@
         <v>46504</v>
       </c>
       <c r="I44" s="14" t="n">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="J44" s="10" t="n">
         <v>46562</v>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="L44" s="9" t="n">
-        <v>0.04941704204942651</v>
+        <v>0.04832803469187192</v>
       </c>
     </row>
     <row r="45">
@@ -2473,7 +2473,7 @@
         <v>46505</v>
       </c>
       <c r="I45" s="21" t="n">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="J45" s="20" t="n">
         <v>46526</v>
@@ -2484,7 +2484,7 @@
         </is>
       </c>
       <c r="L45" s="19" t="n">
-        <v>0.01903762580466897</v>
+        <v>0.01786279313034211</v>
       </c>
     </row>
     <row r="46">
@@ -2519,7 +2519,7 @@
         <v>46508</v>
       </c>
       <c r="I46" s="14" t="n">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="J46" s="10" t="n">
         <v>46518</v>
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="L46" s="9" t="n">
-        <v>0.04781997143077665</v>
+        <v>0.04579785550402819</v>
       </c>
     </row>
     <row r="47">
@@ -2565,7 +2565,7 @@
         <v>46515</v>
       </c>
       <c r="I47" s="14" t="n">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="J47" s="10" t="n">
         <v>46542</v>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="L47" s="9" t="n">
-        <v>0.04754065390450687</v>
+        <v>0.04691896062464589</v>
       </c>
     </row>
     <row r="48">
@@ -2611,7 +2611,7 @@
         <v>46532</v>
       </c>
       <c r="I48" s="14" t="n">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="J48" s="10" t="n">
         <v>46563</v>
@@ -2622,7 +2622,7 @@
         </is>
       </c>
       <c r="L48" s="9" t="n">
-        <v>0.03316635032377153</v>
+        <v>0.03109143998051593</v>
       </c>
     </row>
     <row r="49">
@@ -2657,7 +2657,7 @@
         <v>46589</v>
       </c>
       <c r="I49" s="14" t="n">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="J49" s="10" t="n">
         <v>46629</v>
@@ -2668,7 +2668,7 @@
         </is>
       </c>
       <c r="L49" s="9" t="n">
-        <v>0.02059799423192274</v>
+        <v>0.02034092608022438</v>
       </c>
     </row>
     <row r="50">
@@ -2703,7 +2703,7 @@
         <v>46591</v>
       </c>
       <c r="I50" s="14" t="n">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="J50" s="10" t="n">
         <v>46633</v>
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="L50" s="9" t="n">
-        <v>0.0376935160759064</v>
+        <v>0.03798756490592253</v>
       </c>
     </row>
     <row r="51">
@@ -2749,7 +2749,7 @@
         <v>46594</v>
       </c>
       <c r="I51" s="14" t="n">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="J51" s="10" t="n">
         <v>46613</v>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="L51" s="9" t="n">
-        <v>0.01569066954036555</v>
+        <v>0.01515180818849923</v>
       </c>
     </row>
     <row r="52">
@@ -2795,7 +2795,7 @@
         <v>46595</v>
       </c>
       <c r="I52" s="14" t="n">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="J52" s="10" t="n">
         <v>46614</v>
@@ -2806,7 +2806,7 @@
         </is>
       </c>
       <c r="L52" s="9" t="n">
-        <v>0.02679754601226994</v>
+        <v>0.02660656666088859</v>
       </c>
     </row>
     <row r="53">
@@ -2841,7 +2841,7 @@
         <v>46597</v>
       </c>
       <c r="I53" s="14" t="n">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="J53" s="10" t="n">
         <v>46611</v>
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="L53" s="9" t="n">
-        <v>0.0615498241205511</v>
+        <v>0.05990893907079166</v>
       </c>
     </row>
     <row r="54">
@@ -2887,7 +2887,7 @@
         <v>46598</v>
       </c>
       <c r="I54" s="14" t="n">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="J54" s="10" t="n">
         <v>46629</v>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.02686576971590722</v>
+        <v>0.02719112911712621</v>
       </c>
     </row>
     <row r="55">
@@ -2933,7 +2933,7 @@
         <v>46614</v>
       </c>
       <c r="I55" s="14" t="n">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="J55" s="10" t="n">
         <v>46662</v>
@@ -2944,7 +2944,7 @@
         </is>
       </c>
       <c r="L55" s="9" t="n">
-        <v>0.03503772989535116</v>
+        <v>0.03471713997023395</v>
       </c>
     </row>
     <row r="56">
@@ -2979,7 +2979,7 @@
         <v>46643</v>
       </c>
       <c r="I56" s="14" t="n">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="J56" s="10" t="n">
         <v>46709</v>
@@ -2990,7 +2990,7 @@
         </is>
       </c>
       <c r="L56" s="9" t="n">
-        <v>0.006893939393939394</v>
+        <v>0.006744487525791792</v>
       </c>
     </row>
     <row r="57">
@@ -3025,7 +3025,7 @@
         <v>46645</v>
       </c>
       <c r="I57" s="14" t="n">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="J57" s="10" t="n">
         <v>46668</v>
@@ -3036,7 +3036,7 @@
         </is>
       </c>
       <c r="L57" s="9" t="n">
-        <v>0.06189487343217447</v>
+        <v>0.06643208841292222</v>
       </c>
     </row>
     <row r="58">
@@ -3071,7 +3071,7 @@
         <v>46650</v>
       </c>
       <c r="I58" s="14" t="n">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="J58" s="10" t="n">
         <v>46690</v>
@@ -3082,7 +3082,7 @@
         </is>
       </c>
       <c r="L58" s="9" t="n">
-        <v>0.0196041137387245</v>
+        <v>0.02024161753504176</v>
       </c>
     </row>
   </sheetData>
@@ -3117,7 +3117,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Expected Increase Announcements by Month - 10/05/2026</t>
+          <t>Expected Increase Announcements by Month - 10/12/2026</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
         <v>46305</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>46339</v>
+        <v>46704</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>0.87</v>
@@ -4175,10 +4175,10 @@
         <v>46665</v>
       </c>
       <c r="D56" s="7" t="n">
-        <v>1.5</v>
+        <v>1.65</v>
       </c>
       <c r="E56" s="8" t="n">
-        <v>0.07142857142857149</v>
+        <v>0.09999999999999994</v>
       </c>
       <c r="F56" s="12" t="inlineStr">
         <is>
@@ -4286,7 +4286,7 @@
         <v>46501</v>
       </c>
       <c r="D62" s="7" t="n">
-        <v>1.125</v>
+        <v>1.084</v>
       </c>
       <c r="E62" s="8" t="n">
         <v>0.03495860165593379</v>
@@ -4900,7 +4900,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Complete Holdings Dividend Summary - 10/05/2026</t>
+          <t>Complete Holdings Dividend Summary - 10/12/2026</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
         <v>1.16</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>0.01000906021484749</v>
+        <v>0.01032212162618396</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>46255</v>
@@ -5057,7 +5057,7 @@
         <v>10.08</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>0.0250733801190597</v>
+        <v>0.02435106070044935</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>46255</v>
@@ -5110,7 +5110,7 @@
         <v>8.552</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>0.004618563878007072</v>
+        <v>0.004833085693226959</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>46231</v>
@@ -5163,7 +5163,7 @@
         <v>2.184</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.02679754601226994</v>
+        <v>0.02660656666088859</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>46251</v>
@@ -5216,7 +5216,7 @@
         <v>2.812</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>0.03974558303886926</v>
+        <v>0.0369854010936235</v>
       </c>
       <c r="I9" s="10" t="n">
         <v>46251</v>
@@ -5269,7 +5269,7 @@
         <v>4.12</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>0.02686576971590722</v>
+        <v>0.02719112911712621</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>46265</v>
@@ -5322,7 +5322,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.0615498241205511</v>
+        <v>0.05990893907079166</v>
       </c>
       <c r="I11" s="10" t="n">
         <v>46246</v>
@@ -5375,7 +5375,7 @@
         <v>5.2</v>
       </c>
       <c r="H12" s="9" t="n">
-        <v>0.01960488686266767</v>
+        <v>0.01841164230021915</v>
       </c>
       <c r="I12" s="10" t="n">
         <v>46274</v>
@@ -5428,7 +5428,7 @@
         <v>0.96</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>0.02546081297917674</v>
+        <v>0.02474864597427012</v>
       </c>
       <c r="I13" s="10" t="n">
         <v>46254</v>
@@ -5481,7 +5481,7 @@
         <v>2.4</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>0.007742684745454336</v>
+        <v>0.007395538275760539</v>
       </c>
       <c r="I14" s="10" t="n">
         <v>46248</v>
@@ -5534,7 +5534,7 @@
         <v>1.68</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>0.01496259367888212</v>
+        <v>0.01454306253370746</v>
       </c>
       <c r="I15" s="10" t="n">
         <v>46297</v>
@@ -5587,7 +5587,7 @@
         <v>7.12</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>0.03491993354817895</v>
+        <v>0.03298357685968453</v>
       </c>
       <c r="I16" s="10" t="n">
         <v>46253</v>
@@ -5640,10 +5640,10 @@
         <v>3.44</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>0.01482915257546235</v>
+        <v>0.01480142827673315</v>
       </c>
       <c r="I17" s="10" t="n">
-        <v>46211</v>
+        <v>46301</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>0.07499999999999993</v>
@@ -5693,7 +5693,7 @@
         <v>1.28</v>
       </c>
       <c r="H18" s="9" t="n">
-        <v>0.02692469447517261</v>
+        <v>0.02608518459263433</v>
       </c>
       <c r="I18" s="10" t="n">
         <v>46280</v>
@@ -5746,7 +5746,7 @@
         <v>3.36</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>0.05169230769230769</v>
+        <v>0.05388501362627859</v>
       </c>
       <c r="I19" s="10" t="n">
         <v>46280</v>
@@ -5799,7 +5799,7 @@
         <v>2.56</v>
       </c>
       <c r="H20" s="9" t="n">
-        <v>0.02542835780877885</v>
+        <v>0.02477139648518534</v>
       </c>
       <c r="I20" s="10" t="n">
         <v>46247</v>
@@ -5852,10 +5852,10 @@
         <v>6.36</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>0.01926572184075763</v>
+        <v>0.01906817724130214</v>
       </c>
       <c r="I21" s="10" t="n">
-        <v>46205</v>
+        <v>46304</v>
       </c>
       <c r="J21" s="8" t="n">
         <v>0.06000000000000005</v>
@@ -5905,7 +5905,7 @@
         <v>1.18</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>0.0152012882447665</v>
+        <v>0.01507024206908392</v>
       </c>
       <c r="I22" s="20" t="n">
         <v>46223</v>
@@ -5958,7 +5958,7 @@
         <v>9.32</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>0.03327086122266845</v>
+        <v>0.03219121426382717</v>
       </c>
       <c r="I23" s="10" t="n">
         <v>46268</v>
@@ -6011,7 +6011,7 @@
         <v>5.52</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>0.02049834685596653</v>
+        <v>0.02065597808138082</v>
       </c>
       <c r="I24" s="10" t="n">
         <v>46262</v>
@@ -6064,7 +6064,7 @@
         <v>1.172</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>0.05796241542035767</v>
+        <v>0.06113719328824217</v>
       </c>
       <c r="I25" s="10" t="n">
         <v>46216</v>
@@ -6117,7 +6117,7 @@
         <v>2</v>
       </c>
       <c r="H26" s="19" t="n">
-        <v>0.0275824016146412</v>
+        <v>0.02748952065840456</v>
       </c>
       <c r="I26" s="20" t="n">
         <v>46269</v>
@@ -6170,7 +6170,7 @@
         <v>3.32</v>
       </c>
       <c r="H27" s="9" t="n">
-        <v>0.03503772989535116</v>
+        <v>0.03471713997023395</v>
       </c>
       <c r="I27" s="10" t="n">
         <v>46296</v>
@@ -6223,7 +6223,7 @@
         <v>2.44</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>0.01707069676200025</v>
+        <v>0.01631015976237089</v>
       </c>
       <c r="I28" s="10" t="n">
         <v>46269</v>
@@ -6276,7 +6276,7 @@
         <v>5.36</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.02101466341764813</v>
+        <v>0.02043461780192916</v>
       </c>
       <c r="I29" s="10" t="n">
         <v>46259</v>
@@ -6323,19 +6323,19 @@
         </is>
       </c>
       <c r="F30" s="7" t="n">
-        <v>1.5</v>
+        <v>1.65</v>
       </c>
       <c r="G30" s="26" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.01813072291056532</v>
+        <v>0.01974688024131375</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>46209</v>
+        <v>46301</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>0.07142857142857149</v>
+        <v>0.09999999999999994</v>
       </c>
       <c r="K30" s="10" t="n">
         <v>46461</v>
@@ -6376,16 +6376,16 @@
         </is>
       </c>
       <c r="F31" s="7" t="n">
-        <v>1.125</v>
+        <v>1.084</v>
       </c>
       <c r="G31" s="26" t="n">
-        <v>2.25</v>
+        <v>2.168</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>0.02102116058315701</v>
+        <v>0.01961369636922693</v>
       </c>
       <c r="I31" s="10" t="n">
-        <v>46216</v>
+        <v>46304</v>
       </c>
       <c r="J31" s="8" t="n">
         <v>0.03495860165593379</v>
@@ -6435,7 +6435,7 @@
         <v>3.16</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.0116302613355222</v>
+        <v>0.01212074758762932</v>
       </c>
       <c r="I32" s="10" t="n">
         <v>46295</v>
@@ -6488,7 +6488,7 @@
         <v>2.88</v>
       </c>
       <c r="H33" s="9" t="n">
-        <v>0.03316635032377153</v>
+        <v>0.03109143998051593</v>
       </c>
       <c r="I33" s="10" t="n">
         <v>46290</v>
@@ -6541,7 +6541,7 @@
         <v>1.92</v>
       </c>
       <c r="H34" s="9" t="n">
-        <v>0.04340945104841216</v>
+        <v>0.04253433819142445</v>
       </c>
       <c r="I34" s="10" t="n">
         <v>46209</v>
@@ -6594,7 +6594,7 @@
         <v>3.64</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>0.006893939393939394</v>
+        <v>0.006744487525791792</v>
       </c>
       <c r="I35" s="10" t="n">
         <v>46254</v>
@@ -6647,7 +6647,7 @@
         <v>3.48</v>
       </c>
       <c r="H36" s="9" t="n">
-        <v>0.0269120722736316</v>
+        <v>0.02696629149713606</v>
       </c>
       <c r="I36" s="10" t="n">
         <v>46211</v>
@@ -6659,7 +6659,7 @@
         <v>46305</v>
       </c>
       <c r="L36" s="10" t="n">
-        <v>46339</v>
+        <v>46704</v>
       </c>
       <c r="M36" s="12" t="inlineStr">
         <is>
@@ -6700,7 +6700,7 @@
         <v>1.64</v>
       </c>
       <c r="H37" s="9" t="n">
-        <v>0.0497045022909573</v>
+        <v>0.04726905935798738</v>
       </c>
       <c r="I37" s="10" t="n">
         <v>46266</v>
@@ -6753,7 +6753,7 @@
         <v>1.158</v>
       </c>
       <c r="H38" s="9" t="n">
-        <v>0.03123398452246422</v>
+        <v>0.03014055323240503</v>
       </c>
       <c r="I38" s="10" t="n">
         <v>46251</v>
@@ -6806,7 +6806,7 @@
         <v>3.264</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>0.06097515550966866</v>
+        <v>0.06026977174155138</v>
       </c>
       <c r="I39" s="10" t="n">
         <v>46295</v>
@@ -6859,7 +6859,7 @@
         <v>4.76</v>
       </c>
       <c r="H40" s="9" t="n">
-        <v>0.04781997143077665</v>
+        <v>0.04579785550402819</v>
       </c>
       <c r="I40" s="10" t="n">
         <v>46231</v>
@@ -6912,7 +6912,7 @@
         <v>2.68</v>
       </c>
       <c r="H41" s="9" t="n">
-        <v>0.03948725344843111</v>
+        <v>0.03777308125827056</v>
       </c>
       <c r="I41" s="10" t="n">
         <v>46274</v>
@@ -6965,7 +6965,7 @@
         <v>5.92</v>
       </c>
       <c r="H42" s="9" t="n">
-        <v>0.04754065390450687</v>
+        <v>0.04691896062464589</v>
       </c>
       <c r="I42" s="10" t="n">
         <v>46269</v>
@@ -7018,7 +7018,7 @@
         <v>1.72</v>
       </c>
       <c r="H43" s="9" t="n">
-        <v>0.06260236491789237</v>
+        <v>0.060584714229587</v>
       </c>
       <c r="I43" s="10" t="n">
         <v>46227</v>
@@ -7071,7 +7071,7 @@
         <v>3.36</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>0.02993185232025556</v>
+        <v>0.03130677936678974</v>
       </c>
       <c r="I44" s="10" t="n">
         <v>46268</v>
@@ -7124,7 +7124,7 @@
         <v>4.356</v>
       </c>
       <c r="H45" s="9" t="n">
-        <v>0.03003827202933425</v>
+        <v>0.02866072298257646</v>
       </c>
       <c r="I45" s="10" t="n">
         <v>46227</v>
@@ -7177,7 +7177,7 @@
         <v>2.204</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>0.04941704204942651</v>
+        <v>0.04832803469187192</v>
       </c>
       <c r="I46" s="10" t="n">
         <v>46290</v>
@@ -7230,7 +7230,7 @@
         <v>5.08</v>
       </c>
       <c r="H47" s="19" t="n">
-        <v>0.01903762580466897</v>
+        <v>0.01786279313034211</v>
       </c>
       <c r="I47" s="20" t="n">
         <v>46252</v>
@@ -7283,7 +7283,7 @@
         <v>3.92</v>
       </c>
       <c r="H48" s="9" t="n">
-        <v>0.01569066954036555</v>
+        <v>0.01515180818849923</v>
       </c>
       <c r="I48" s="10" t="n">
         <v>46252</v>
@@ -7336,7 +7336,7 @@
         <v>9.76</v>
       </c>
       <c r="H49" s="9" t="n">
-        <v>0.02675878779765391</v>
+        <v>0.0270262782600054</v>
       </c>
       <c r="I49" s="10" t="n">
         <v>46253</v>
@@ -7389,7 +7389,7 @@
         <v>3.36</v>
       </c>
       <c r="H50" s="9" t="n">
-        <v>0.0376935160759064</v>
+        <v>0.03798756490592253</v>
       </c>
       <c r="I50" s="10" t="n">
         <v>46273</v>
@@ -7442,7 +7442,7 @@
         <v>5.2</v>
       </c>
       <c r="H51" s="9" t="n">
-        <v>0.05039736368113923</v>
+        <v>0.05061812352845635</v>
       </c>
       <c r="I51" s="10" t="n">
         <v>46280</v>
@@ -7495,7 +7495,7 @@
         <v>4.084</v>
       </c>
       <c r="H52" s="9" t="n">
-        <v>0.04847765287972164</v>
+        <v>0.04612083409655995</v>
       </c>
       <c r="I52" s="10" t="n">
         <v>46295</v>
@@ -7548,7 +7548,7 @@
         <v>5.68</v>
       </c>
       <c r="H53" s="9" t="n">
-        <v>0.0196041137387245</v>
+        <v>0.02024161753504176</v>
       </c>
       <c r="I53" s="10" t="n">
         <v>46234</v>
@@ -7601,7 +7601,7 @@
         <v>2.124</v>
       </c>
       <c r="H54" s="9" t="n">
-        <v>0.03558086960144769</v>
+        <v>0.03395140590432928</v>
       </c>
       <c r="I54" s="10" t="n">
         <v>46241</v>
@@ -7654,7 +7654,7 @@
         <v>5.68</v>
       </c>
       <c r="H55" s="9" t="n">
-        <v>0.02059799423192274</v>
+        <v>0.02034092608022438</v>
       </c>
       <c r="I55" s="10" t="n">
         <v>46265</v>
@@ -7707,10 +7707,10 @@
         <v>2.832</v>
       </c>
       <c r="H56" s="9" t="n">
-        <v>0.06189487343217447</v>
+        <v>0.06643208841292222</v>
       </c>
       <c r="I56" s="10" t="n">
-        <v>46213</v>
+        <v>46304</v>
       </c>
       <c r="J56" s="8" t="n">
         <v>0.02608695652173916</v>
@@ -7760,7 +7760,7 @@
         <v>4.12</v>
       </c>
       <c r="H57" s="9" t="n">
-        <v>0.025221915188599</v>
+        <v>0.02392427756445954</v>
       </c>
       <c r="I57" s="10" t="n">
         <v>46251</v>

</xml_diff>